<commit_message>
Article « NEP 911 et 912 révisées » en relecture (noindex) : texte, visuels, cartes hub et série
Brief P011 passé en relecture ; correctif du pré-remplissage du <title> dans
new-article.py --brief.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content-plan/plan-editorial.xlsx
+++ b/content-plan/plan-editorial.xlsx
@@ -19,9 +19,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Calendrier'!$A$1:$AA$105</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Piliers'!$A$1:$N$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Requêtes'!$A$1:$H$29</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Distribution'!$A$1:$I$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Distribution'!$A$1:$I$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Suivi IA'!$A$1:$H$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Backlog'!$A$1:$G$92</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Backlog'!$A$1:$G$91</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Légende'!$A$1:$C$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -43,7 +43,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -65,6 +65,11 @@
         <fgColor rgb="00EEEEEE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE699"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -78,7 +83,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -86,6 +91,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1588,9 +1594,9 @@
           <t>P011</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>Idée</t>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Relecture humaine</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1622,7 +1628,7 @@
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Cofondateur commissaire aux comptes (nom à confirmer)</t>
+          <t>L'équipe CheckIA</t>
         </is>
       </c>
       <c r="K12" t="inlineStr"/>
@@ -1645,7 +1651,7 @@
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>JD</t>
+          <t>Chloe</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
@@ -1656,7 +1662,7 @@
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
-          <t>Auteur CAC nommé (nom, titre, LinkedIn) — non</t>
+          <t>Auteur CAC nommé (nom, titre, LinkedIn) — ok (décision Chloe : signature L'équipe CheckIA)</t>
         </is>
       </c>
       <c r="U12" t="inlineStr"/>
@@ -1675,7 +1681,7 @@
       </c>
       <c r="AA12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>non</t>
         </is>
       </c>
     </row>
@@ -11325,7 +11331,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Idée</t>
+          <t>Relecture humaine</t>
         </is>
       </c>
     </row>
@@ -13085,14 +13091,14 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Idée</t>
+          <t>Relecture humaine</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>oui</t>
         </is>
       </c>
     </row>
@@ -13856,7 +13862,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -13944,8 +13950,31 @@
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>P011</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>NEP 911 et 912 révisées (arrêté du 24 juillet 2026) : ce qui change pour les petites entreprises</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://checkia.fr/blog/futur-de-l-audit/nep-911-912-revisees-2026/</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I2"/>
+  <autoFilter ref="A1:I3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -14050,7 +14079,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G92"/>
+  <dimension ref="A1:G91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -14382,7 +14411,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>P011</t>
+          <t>P012</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
@@ -14392,12 +14421,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>NEP 911 et 912 révisées (arrêté du 24 juillet 2026) : ce qui change pour les petites entreprises</t>
+          <t>Panorama des logiciels pour commissaires aux comptes 2026</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>P1b NEP</t>
+          <t>P3 Logiciel CAC</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -14407,19 +14436,15 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>JD</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Auteur CAC nommé (nom, titre, LinkedIn) — non</t>
-        </is>
-      </c>
+          <t>Chloe</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>P012</t>
+          <t>P013</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -14429,12 +14454,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Panorama des logiciels pour commissaires aux comptes 2026</t>
+          <t>Charte IA d'un cabinet de commissariat aux comptes : modèle et dix clauses</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>P3 Logiciel CAC</t>
+          <t>P1 IA et CAC</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -14444,15 +14469,19 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Chloe</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr"/>
+          <t>JD</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Auteur CAC nommé (nom, titre, LinkedIn) — non</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>P013</t>
+          <t>P014</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
@@ -14462,17 +14491,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Charte IA d'un cabinet de commissariat aux comptes : modèle et dix clauses</t>
+          <t>Rapport du commissaire aux apports : structure, mentions obligatoires, exemple</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>P1 IA et CAC</t>
+          <t>P2 Missions spécifiques</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>haute</t>
+          <t>normale</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -14489,7 +14518,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>P014</t>
+          <t>P015</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -14499,7 +14528,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Rapport du commissaire aux apports : structure, mentions obligatoires, exemple</t>
+          <t>Lettre de mission du commissaire aux apports : ce qu'elle doit contenir</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -14514,19 +14543,15 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>JD</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Auteur CAC nommé (nom, titre, LinkedIn) — non</t>
-        </is>
-      </c>
+          <t>Chloe</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>P015</t>
+          <t>P016</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
@@ -14536,12 +14561,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Lettre de mission du commissaire aux apports : ce qu'elle doit contenir</t>
+          <t>L'IA va-t-elle remplacer le commissaire aux comptes ?</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>P2 Missions spécifiques</t>
+          <t>P1 IA et CAC</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -14551,15 +14576,19 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Chloe</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr"/>
+          <t>JD</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Auteur CAC nommé (nom, titre, LinkedIn) — non</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>P016</t>
+          <t>P017</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -14569,12 +14598,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>L'IA va-t-elle remplacer le commissaire aux comptes ?</t>
+          <t>Historique des validations : qui a validé quoi, et quand</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>P1 IA et CAC</t>
+          <t>P5 Produit</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -14584,19 +14613,15 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>JD</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Auteur CAC nommé (nom, titre, LinkedIn) — non</t>
-        </is>
-      </c>
+          <t>Chloe</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>P017</t>
+          <t>P018</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
@@ -14606,12 +14631,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Historique des validations : qui a validé quoi, et quand</t>
+          <t>Ce que l'IA peut et ne peut pas faire dans un dossier : entretien avec Jean-David Collard, docteur en IA</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>P5 Produit</t>
+          <t>P4 Paroles de CAC</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -14624,12 +14649,16 @@
           <t>Chloe</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Citations validées par l'interviewé — non</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>P018</t>
+          <t>P019</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
@@ -14639,12 +14668,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Ce que l'IA peut et ne peut pas faire dans un dossier : entretien avec Jean-David Collard, docteur en IA</t>
+          <t>Combien coûte un logiciel de commissariat aux comptes ?</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>P4 Paroles de CAC</t>
+          <t>P3 Logiciel CAC</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -14659,14 +14688,14 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Citations validées par l'interviewé — non</t>
+          <t>Position de CheckIA sur la publication d'un prix — non</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>P019</t>
+          <t>P020</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
@@ -14676,17 +14705,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Combien coûte un logiciel de commissariat aux comptes ?</t>
+          <t>Lancement de l'enquête « Baromètre de la formalisation » auprès des commissaires aux comptes</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>P3 Logiciel CAC</t>
+          <t>Hors site</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>normale</t>
+          <t>haute</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -14694,16 +14723,12 @@
           <t>Chloe</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Position de CheckIA sur la publication d'un prix — non</t>
-        </is>
-      </c>
+      <c r="G18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>P020</t>
+          <t>P021</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
@@ -14713,30 +14738,34 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Lancement de l'enquête « Baromètre de la formalisation » auprès des commissaires aux comptes</t>
+          <t>Seuil de signification (NEP 320) : calcul, seuils de planification et documentation</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Hors site</t>
+          <t>P1b NEP</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>haute</t>
+          <t>normale</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Chloe</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr"/>
+          <t>JD</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Auteur CAC nommé (nom, titre, LinkedIn) — non</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>P021</t>
+          <t>P022</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
@@ -14746,17 +14775,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Seuil de signification (NEP 320) : calcul, seuils de planification et documentation</t>
+          <t>Secret professionnel du commissaire aux comptes et IA : ce que permet l'article L. 821-35</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>P1b NEP</t>
+          <t>P1 IA et CAC</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>normale</t>
+          <t>haute</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -14773,7 +14802,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>P022</t>
+          <t>P023</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
@@ -14783,7 +14812,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Secret professionnel du commissaire aux comptes et IA : ce que permet l'article L. 821-35</t>
+          <t>AI Act et cabinets d'audit : l'obligation de littératie IA depuis le 2 août 2026</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -14793,7 +14822,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>haute</t>
+          <t>normale</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -14810,7 +14839,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>P023</t>
+          <t>P024</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
@@ -14820,7 +14849,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>AI Act et cabinets d'audit : l'obligation de littératie IA depuis le 2 août 2026</t>
+          <t>L'IA comme un collaborateur à superviser : la position de la H2A (juillet 2026)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -14835,19 +14864,15 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>JD</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Auteur CAC nommé (nom, titre, LinkedIn) — non</t>
-        </is>
-      </c>
+          <t>Chloe</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>P024</t>
+          <t>P025</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
@@ -14857,12 +14882,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>L'IA comme un collaborateur à superviser : la position de la H2A (juillet 2026)</t>
+          <t>Nomination du commissaire aux apports : unanimité des associés ou ordonnance sur requête ?</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>P1 IA et CAC</t>
+          <t>P2 Missions spécifiques</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -14872,15 +14897,19 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Chloe</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr"/>
+          <t>JD</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Auteur CAC nommé (nom, titre, LinkedIn) — non</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>P025</t>
+          <t>P026</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
@@ -14890,7 +14919,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Nomination du commissaire aux apports : unanimité des associés ou ordonnance sur requête ?</t>
+          <t>Commissaire aux apports et auto-révision : les cas à refuser</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -14917,7 +14946,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>P026</t>
+          <t>P027</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
@@ -14927,12 +14956,12 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Commissaire aux apports et auto-révision : les cas à refuser</t>
+          <t>Éditeur DOCX natif et export PDF : relire et corriger sans quitter le dossier</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>P2 Missions spécifiques</t>
+          <t>P5 Produit</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -14942,19 +14971,15 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>JD</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>Auteur CAC nommé (nom, titre, LinkedIn) — non</t>
-        </is>
-      </c>
+          <t>Chloe</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>P027</t>
+          <t>P028</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
@@ -14964,12 +14989,12 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Éditeur DOCX natif et export PDF : relire et corriger sans quitter le dossier</t>
+          <t>L'IA dans un cabinet de commissaires aux comptes : entretien avec un praticien</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>P5 Produit</t>
+          <t>P4 Paroles de CAC</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -14982,12 +15007,16 @@
           <t>Chloe</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Interviewé confirmé — non ; Citations validées par l'interviewé — non</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>P028</t>
+          <t>P029</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
@@ -14997,12 +15026,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>L'IA dans un cabinet de commissaires aux comptes : entretien avec un praticien</t>
+          <t>Quel logiciel pour les missions spécifiques du commissaire aux comptes ?</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>P4 Paroles de CAC</t>
+          <t>P3 Logiciel CAC</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -15015,16 +15044,12 @@
           <t>Chloe</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>Interviewé confirmé — non ; Citations validées par l'interviewé — non</t>
-        </is>
-      </c>
+      <c r="G27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>P029</t>
+          <t>P030</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
@@ -15034,12 +15059,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Quel logiciel pour les missions spécifiques du commissaire aux comptes ?</t>
+          <t>Plan de mission (NEP 300) : structure, contenu et modèle</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>P3 Logiciel CAC</t>
+          <t>P1b NEP</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -15049,15 +15074,19 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Chloe</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr"/>
+          <t>JD</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Auteur CAC nommé (nom, titre, LinkedIn) — non</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>P030</t>
+          <t>P031</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
@@ -15067,34 +15096,34 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Plan de mission (NEP 300) : structure, contenu et modèle</t>
+          <t>Assises 2026 « IA : Innovation et Audit » : ce que nous en retenons</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>P1b NEP</t>
+          <t>P1 IA et CAC</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>normale</t>
+          <t>haute</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>JD</t>
+          <t>Chloe</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Auteur CAC nommé (nom, titre, LinkedIn) — non</t>
+          <t>Présence aux Assises confirmée — non</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>P031</t>
+          <t>P032</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
@@ -15104,12 +15133,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Assises 2026 « IA : Innovation et Audit » : ce que nous en retenons</t>
+          <t>NEP 315 et outils et techniques automatisés : comment documenter l'usage de l'IA</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>P1 IA et CAC</t>
+          <t>P1b NEP</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -15119,19 +15148,19 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Chloe</t>
+          <t>JD</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Présence aux Assises confirmée — non</t>
+          <t>Auteur CAC nommé (nom, titre, LinkedIn) — non</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>P032</t>
+          <t>P033</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
@@ -15141,17 +15170,17 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>NEP 315 et outils et techniques automatisés : comment documenter l'usage de l'IA</t>
+          <t>Fusion-absorption d'une SCI par une SAS : faut-il un commissaire aux apports ?</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>P1b NEP</t>
+          <t>P2 Missions spécifiques</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>haute</t>
+          <t>normale</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -15168,7 +15197,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>P033</t>
+          <t>P034</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
@@ -15178,7 +15207,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Fusion-absorption d'une SCI par une SAS : faut-il un commissaire aux apports ?</t>
+          <t>Apports en fin d'année : calendrier et pièces à réunir avant le 31 décembre</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -15193,19 +15222,15 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>JD</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>Auteur CAC nommé (nom, titre, LinkedIn) — non</t>
-        </is>
-      </c>
+          <t>Chloe</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>P034</t>
+          <t>P035</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
@@ -15215,12 +15240,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Apports en fin d'année : calendrier et pièces à réunir avant le 31 décembre</t>
+          <t>[IA] Première fonctionnalité d'assistance par IA dans CheckIA (titre à préciser au lancement)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>P2 Missions spécifiques</t>
+          <t>P5 Produit</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -15233,12 +15258,16 @@
           <t>Chloe</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Fonctionnalité IA en production — non ; produit-verite.md mis à jour ([ia-assistance] déplacé en production, [aucune-ia-externe] réévalué) — non</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>P035</t>
+          <t>P036</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
@@ -15248,12 +15277,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>[IA] Première fonctionnalité d'assistance par IA dans CheckIA (titre à préciser au lancement)</t>
+          <t>[Cabinet] : [résultat obtenu avec CheckIA] — premier témoignage client</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>P5 Produit</t>
+          <t>P4 Paroles de CAC</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -15268,14 +15297,14 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Fonctionnalité IA en production — non ; produit-verite.md mis à jour ([ia-assistance] déplacé en production, [aucune-ia-externe] réévalué) — non</t>
+          <t>Cabinet client volontaire identifié — non ; Citations validées par l'interviewé — non</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>P036</t>
+          <t>P037</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
@@ -15285,12 +15314,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>[Cabinet] : [résultat obtenu avec CheckIA] — premier témoignage client</t>
+          <t>CheckIA en 2026 : bilan et feuille de route 2027</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>P4 Paroles de CAC</t>
+          <t>P6 Entreprise</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -15303,16 +15332,12 @@
           <t>Chloe</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>Cabinet client volontaire identifié — non ; Citations validées par l'interviewé — non</t>
-        </is>
-      </c>
+      <c r="G35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>P037</t>
+          <t>P038</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
@@ -15322,30 +15347,34 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>CheckIA en 2026 : bilan et feuille de route 2027</t>
+          <t>Baromètre de la formalisation 2027 : combien de temps les commissaires aux comptes passent-ils à formaliser ?</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>P6 Entreprise</t>
+          <t>P1 IA et CAC</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>normale</t>
+          <t>haute</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Chloe</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr"/>
+          <t>JD</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Au moins 100 réponses collectées — non ; Auteur CAC nommé (nom, titre, LinkedIn) — non</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>P038</t>
+          <t>P039</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
@@ -15355,17 +15384,17 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Baromètre de la formalisation 2027 : combien de temps les commissaires aux comptes passent-ils à formaliser ?</t>
+          <t>NEP 230 : ce qu'un dossier de mission spécifique doit contenir pour être compréhensible sans explication orale</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>P1 IA et CAC</t>
+          <t>P1b NEP</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>haute</t>
+          <t>normale</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -15375,14 +15404,14 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Au moins 100 réponses collectées — non ; Auteur CAC nommé (nom, titre, LinkedIn) — non</t>
+          <t>Auteur CAC nommé (nom, titre, LinkedIn) — non</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>P039</t>
+          <t>P040</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
@@ -15392,17 +15421,17 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>NEP 230 : ce qu'un dossier de mission spécifique doit contenir pour être compréhensible sans explication orale</t>
+          <t>Commissariat à la transformation : procédure, rapport et délai de huit jours (L. 224-3)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>P1b NEP</t>
+          <t>P2 Missions spécifiques</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>normale</t>
+          <t>haute</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -15419,7 +15448,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>P040</t>
+          <t>P041</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
@@ -15429,7 +15458,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Commissariat à la transformation : procédure, rapport et délai de huit jours (L. 224-3)</t>
+          <t>Transformation en société par actions : quand faut-il un commissaire à la transformation ?</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -15439,24 +15468,20 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>haute</t>
+          <t>normale</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>JD</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>Auteur CAC nommé (nom, titre, LinkedIn) — non</t>
-        </is>
-      </c>
+          <t>Chloe</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>P041</t>
+          <t>P042</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
@@ -15466,12 +15491,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Transformation en société par actions : quand faut-il un commissaire à la transformation ?</t>
+          <t>Excel et Word pour les missions spécifiques : les limites et le moment de changer</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>P2 Missions spécifiques</t>
+          <t>P3 Logiciel CAC</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -15489,7 +15514,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>P042</t>
+          <t>P043</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
@@ -15499,12 +15524,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Excel et Word pour les missions spécifiques : les limites et le moment de changer</t>
+          <t>Nouveautés produit de janvier 2027 (à préciser depuis le journal de développement)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>P3 Logiciel CAC</t>
+          <t>P5 Produit</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -15517,12 +15542,16 @@
           <t>Chloe</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr"/>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Fonctionnalités du mois identifiées et ajoutées à produit-verite.md — non</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>P043</t>
+          <t>P044</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
@@ -15532,12 +15561,12 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Nouveautés produit de janvier 2027 (à préciser depuis le journal de développement)</t>
+          <t>Paroles de commissaires aux comptes n° 4 (invité à confirmer)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>P5 Produit</t>
+          <t>P4 Paroles de CAC</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -15552,14 +15581,14 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Fonctionnalités du mois identifiées et ajoutées à produit-verite.md — non</t>
+          <t>Interviewé confirmé — non</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>P044</t>
+          <t>P045</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
@@ -15569,12 +15598,12 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Paroles de commissaires aux comptes n° 4 (invité à confirmer)</t>
+          <t>Rafraîchissement trimestriel du panorama des logiciels CAC (T1 2027)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>P4 Paroles de CAC</t>
+          <t>P3 Logiciel CAC</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -15587,16 +15616,12 @@
           <t>Chloe</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>Interviewé confirmé — non</t>
-        </is>
-      </c>
+      <c r="G43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>P045</t>
+          <t>P046</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
@@ -15606,12 +15631,12 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Rafraîchissement trimestriel du panorama des logiciels CAC (T1 2027)</t>
+          <t>Produire un texte n'est pas documenter une mission : pourquoi le prompting ne remplace pas le dossier</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>P3 Logiciel CAC</t>
+          <t>P1 IA et CAC</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -15621,15 +15646,19 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Chloe</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr"/>
+          <t>JD</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Auteur CAC nommé (nom, titre, LinkedIn) — non</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>P046</t>
+          <t>P047</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
@@ -15639,7 +15668,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Produire un texte n'est pas documenter une mission : pourquoi le prompting ne remplace pas le dossier</t>
+          <t>Piste d'audit des décisions humaines et de l'IA : proposition, validation, modification</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -15654,19 +15683,15 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>JD</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>Auteur CAC nommé (nom, titre, LinkedIn) — non</t>
-        </is>
-      </c>
+          <t>Chloe</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>P047</t>
+          <t>P048</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
@@ -15676,12 +15701,12 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Piste d'audit des décisions humaines et de l'IA : proposition, validation, modification</t>
+          <t>Évaluation des apports : méthodes retenues et justification dans le rapport</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>P1 IA et CAC</t>
+          <t>P2 Missions spécifiques</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -15691,15 +15716,19 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Chloe</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr"/>
+          <t>JD</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Auteur CAC nommé (nom, titre, LinkedIn) — non</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>P048</t>
+          <t>P049</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
@@ -15709,7 +15738,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Évaluation des apports : méthodes retenues et justification dans le rapport</t>
+          <t>Avantages particuliers : ce que vérifie le commissaire aux apports ou à la transformation</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -15736,7 +15765,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>P049</t>
+          <t>P050</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
@@ -15746,12 +15775,12 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Avantages particuliers : ce que vérifie le commissaire aux apports ou à la transformation</t>
+          <t>Migrer ses dossiers vers un logiciel CAC : formats, conservation et contrôles de reprise</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>P2 Missions spécifiques</t>
+          <t>P3 Logiciel CAC</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -15761,19 +15790,15 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>JD</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>Auteur CAC nommé (nom, titre, LinkedIn) — non</t>
-        </is>
-      </c>
+          <t>Chloe</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>P050</t>
+          <t>P051</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
@@ -15783,12 +15808,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Migrer ses dossiers vers un logiciel CAC : formats, conservation et contrôles de reprise</t>
+          <t>Nouveautés produit de février 2027 (à préciser)</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>P3 Logiciel CAC</t>
+          <t>P5 Produit</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -15801,12 +15826,16 @@
           <t>Chloe</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr"/>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Fonctionnalités du mois identifiées — non</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>P051</t>
+          <t>P052</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
@@ -15816,12 +15845,12 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Nouveautés produit de février 2027 (à préciser)</t>
+          <t>Paroles de commissaires aux comptes n° 5 (invité à confirmer)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>P5 Produit</t>
+          <t>P4 Paroles de CAC</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -15836,14 +15865,14 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Fonctionnalités du mois identifiées — non</t>
+          <t>Interviewé confirmé — non</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>P052</t>
+          <t>P053</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
@@ -15853,7 +15882,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Paroles de commissaires aux comptes n° 5 (invité à confirmer)</t>
+          <t>Deuxième témoignage client (cabinet à confirmer)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -15873,14 +15902,14 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Interviewé confirmé — non</t>
+          <t>Cabinet client volontaire identifié — non</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>P053</t>
+          <t>P054</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
@@ -15890,12 +15919,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Deuxième témoignage client (cabinet à confirmer)</t>
+          <t>Journée Confiance Numérique 2027 : ce que la CNCC a annoncé sur l'IA</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>P4 Paroles de CAC</t>
+          <t>P1 IA et CAC</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -15910,14 +15939,14 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Cabinet client volontaire identifié — non</t>
+          <t>Présence confirmée — non</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>P054</t>
+          <t>P055</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
@@ -15927,7 +15956,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Journée Confiance Numérique 2027 : ce que la CNCC a annoncé sur l'IA</t>
+          <t>Omnibus et CSRD : ce qui change pour le commissaire aux comptes en France (2027)</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -15942,19 +15971,19 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Chloe</t>
+          <t>JD</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Présence confirmée — non</t>
+          <t>Auteur CAC nommé (nom, titre, LinkedIn) — non</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>P055</t>
+          <t>P056</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
@@ -15964,7 +15993,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Omnibus et CSRD : ce qui change pour le commissaire aux comptes en France (2027)</t>
+          <t>Contrôle d'activité H2A : comment prouver un usage encadré de l'IA</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -15991,7 +16020,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>P056</t>
+          <t>P057</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
@@ -16001,12 +16030,12 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Contrôle d'activité H2A : comment prouver un usage encadré de l'IA</t>
+          <t>Fiche d'acceptation et attestation d'indépendance en mission spécifique</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>P1 IA et CAC</t>
+          <t>P2 Missions spécifiques</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -16016,19 +16045,15 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>JD</t>
-        </is>
-      </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>Auteur CAC nommé (nom, titre, LinkedIn) — non</t>
-        </is>
-      </c>
+          <t>Chloe</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>P057</t>
+          <t>P058</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
@@ -16038,12 +16063,12 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Fiche d'acceptation et attestation d'indépendance en mission spécifique</t>
+          <t>Adopter un logiciel CAC en 30, 60 et 90 jours : plan pour les associés</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>P2 Missions spécifiques</t>
+          <t>P3 Logiciel CAC</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -16061,7 +16086,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>P058</t>
+          <t>P059</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
@@ -16071,12 +16096,12 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Adopter un logiciel CAC en 30, 60 et 90 jours : plan pour les associés</t>
+          <t>Nouveautés produit de mars 2027 (à préciser)</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>P3 Logiciel CAC</t>
+          <t>P5 Produit</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -16089,12 +16114,16 @@
           <t>Chloe</t>
         </is>
       </c>
-      <c r="G57" t="inlineStr"/>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Fonctionnalités du mois identifiées — non</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>P059</t>
+          <t>P060</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
@@ -16104,12 +16133,12 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Nouveautés produit de mars 2027 (à préciser)</t>
+          <t>Paroles de commissaires aux comptes n° 6 (invité à confirmer)</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>P5 Produit</t>
+          <t>P4 Paroles de CAC</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -16124,14 +16153,14 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Fonctionnalités du mois identifiées — non</t>
+          <t>Interviewé confirmé — non</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>P060</t>
+          <t>P061</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
@@ -16141,12 +16170,12 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Paroles de commissaires aux comptes n° 6 (invité à confirmer)</t>
+          <t>Rafraîchissement du guide « IA et commissariat aux comptes » après la Journée Confiance Numérique</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>P4 Paroles de CAC</t>
+          <t>P1 IA et CAC</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -16159,16 +16188,12 @@
           <t>Chloe</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>Interviewé confirmé — non</t>
-        </is>
-      </c>
+      <c r="G59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>P061</t>
+          <t>P062</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
@@ -16178,12 +16203,12 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Rafraîchissement du guide « IA et commissariat aux comptes » après la Journée Confiance Numérique</t>
+          <t>Honoraires du commissaire aux apports : repères 2027</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>P1 IA et CAC</t>
+          <t>P2 Missions spécifiques</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -16193,15 +16218,19 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Chloe</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr"/>
+          <t>JD</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Auteur CAC nommé (nom, titre, LinkedIn) — non</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>P062</t>
+          <t>P063</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
@@ -16211,7 +16240,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Honoraires du commissaire aux apports : repères 2027</t>
+          <t>Apport en nature et apport de titres : différences pratiques pour le commissaire aux apports</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -16238,7 +16267,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>P063</t>
+          <t>P064</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
@@ -16248,12 +16277,12 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Apport en nature et apport de titres : différences pratiques pour le commissaire aux apports</t>
+          <t>Les prompts à éviter en cabinet de commissaires aux comptes, et leurs alternatives</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>P2 Missions spécifiques</t>
+          <t>P1 IA et CAC</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -16263,19 +16292,15 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>JD</t>
-        </is>
-      </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>Auteur CAC nommé (nom, titre, LinkedIn) — non</t>
-        </is>
-      </c>
+          <t>Chloe</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>P064</t>
+          <t>P065</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
@@ -16285,12 +16310,12 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Les prompts à éviter en cabinet de commissaires aux comptes, et leurs alternatives</t>
+          <t>Logiciel dédié ou suite bureautique avec IA générique : comparatif pour les missions spécifiques</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>P1 IA et CAC</t>
+          <t>P3 Logiciel CAC</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -16308,7 +16333,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>P065</t>
+          <t>P066</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
@@ -16318,12 +16343,12 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Logiciel dédié ou suite bureautique avec IA générique : comparatif pour les missions spécifiques</t>
+          <t>Nouveautés produit d'avril 2027 (à préciser)</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>P3 Logiciel CAC</t>
+          <t>P5 Produit</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -16336,12 +16361,16 @@
           <t>Chloe</t>
         </is>
       </c>
-      <c r="G64" t="inlineStr"/>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Fonctionnalités du mois identifiées — non</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>P066</t>
+          <t>P067</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
@@ -16351,12 +16380,12 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Nouveautés produit d'avril 2027 (à préciser)</t>
+          <t>Paroles de commissaires aux comptes n° 7 : apports et créateurs d'entreprise (GO Entrepreneurs)</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>P5 Produit</t>
+          <t>P4 Paroles de CAC</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -16371,14 +16400,14 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Fonctionnalités du mois identifiées — non</t>
+          <t>Interviewé confirmé — non</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>P067</t>
+          <t>P068</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
@@ -16388,7 +16417,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Paroles de commissaires aux comptes n° 7 : apports et créateurs d'entreprise (GO Entrepreneurs)</t>
+          <t>Troisième témoignage client (cabinet à confirmer)</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -16408,14 +16437,14 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Interviewé confirmé — non</t>
+          <t>Cabinet client volontaire identifié — non</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>P068</t>
+          <t>P069</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
@@ -16425,12 +16454,12 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Troisième témoignage client (cabinet à confirmer)</t>
+          <t>Rafraîchissement de deux articles de 2026 (à choisir selon le suivi des citations)</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>P4 Paroles de CAC</t>
+          <t>P1 IA et CAC</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -16443,16 +16472,12 @@
           <t>Chloe</t>
         </is>
       </c>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t>Cabinet client volontaire identifié — non</t>
-        </is>
-      </c>
+      <c r="G67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>P069</t>
+          <t>P070</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
@@ -16462,12 +16487,12 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Rafraîchissement de deux articles de 2026 (à choisir selon le suivi des citations)</t>
+          <t>Checklist du dossier de commissariat aux apports : les points à vérifier avant archivage</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>P1 IA et CAC</t>
+          <t>P2 Missions spécifiques</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -16485,7 +16510,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>P070</t>
+          <t>P071</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
@@ -16495,7 +16520,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Checklist du dossier de commissariat aux apports : les points à vérifier avant archivage</t>
+          <t>Lettre d'affirmation en mission spécifique : rôle, contenu et moment de signature</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -16510,15 +16535,19 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Chloe</t>
-        </is>
-      </c>
-      <c r="G69" t="inlineStr"/>
+          <t>JD</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Auteur CAC nommé (nom, titre, LinkedIn) — non</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>P071</t>
+          <t>P072</t>
         </is>
       </c>
       <c r="B70" s="4" t="inlineStr">
@@ -16528,12 +16557,12 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Lettre d'affirmation en mission spécifique : rôle, contenu et moment de signature</t>
+          <t>Former ses collaborateurs à l'IA : plan de formation et preuves à conserver</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>P2 Missions spécifiques</t>
+          <t>P1 IA et CAC</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -16543,19 +16572,15 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>JD</t>
-        </is>
-      </c>
-      <c r="G70" t="inlineStr">
-        <is>
-          <t>Auteur CAC nommé (nom, titre, LinkedIn) — non</t>
-        </is>
-      </c>
+          <t>Chloe</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>P072</t>
+          <t>P073</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr">
@@ -16565,12 +16590,12 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Former ses collaborateurs à l'IA : plan de formation et preuves à conserver</t>
+          <t>Nouveautés produit de mai 2027 (à préciser)</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>P1 IA et CAC</t>
+          <t>P5 Produit</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -16583,12 +16608,16 @@
           <t>Chloe</t>
         </is>
       </c>
-      <c r="G71" t="inlineStr"/>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Fonctionnalités du mois identifiées — non</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>P073</t>
+          <t>P074</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">
@@ -16598,12 +16627,12 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Nouveautés produit de mai 2027 (à préciser)</t>
+          <t>Paroles de commissaires aux comptes n° 8 (invité à confirmer)</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>P5 Produit</t>
+          <t>P4 Paroles de CAC</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -16618,14 +16647,14 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Fonctionnalités du mois identifiées — non</t>
+          <t>Interviewé confirmé — non</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>P074</t>
+          <t>P075</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
@@ -16635,12 +16664,12 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Paroles de commissaires aux comptes n° 8 (invité à confirmer)</t>
+          <t>Rafraîchissement du guide « Commissariat aux apports » et d'un article NEP</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>P4 Paroles de CAC</t>
+          <t>P2 Missions spécifiques</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -16653,16 +16682,12 @@
           <t>Chloe</t>
         </is>
       </c>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>Interviewé confirmé — non</t>
-        </is>
-      </c>
+      <c r="G73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>P075</t>
+          <t>P076</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
@@ -16672,12 +16697,12 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Rafraîchissement du guide « Commissariat aux apports » et d'un article NEP</t>
+          <t>Rafraîchissement de l'article NEP 911/912 après un an d'application</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>P2 Missions spécifiques</t>
+          <t>P1b NEP</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -16695,7 +16720,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>P076</t>
+          <t>P077</t>
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr">
@@ -16705,12 +16730,12 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Rafraîchissement de l'article NEP 911/912 après un an d'application</t>
+          <t>Baromètre CNCC 2027 : ce que les chiffres disent aux cabinets</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>P1b NEP</t>
+          <t>P1 IA et CAC</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -16720,15 +16745,19 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Chloe</t>
-        </is>
-      </c>
-      <c r="G75" t="inlineStr"/>
+          <t>JD</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Baromètre CNCC 2027 publié — non ; Auteur CAC nommé (nom, titre, LinkedIn) — non</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>P077</t>
+          <t>P078</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
@@ -16738,12 +16767,12 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Baromètre CNCC 2027 : ce que les chiffres disent aux cabinets</t>
+          <t>Assemblée du 30 juin : ce que le commissaire à la transformation doit avoir remis huit jours avant</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>P1 IA et CAC</t>
+          <t>P2 Missions spécifiques</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -16753,19 +16782,15 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>JD</t>
-        </is>
-      </c>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>Baromètre CNCC 2027 publié — non ; Auteur CAC nommé (nom, titre, LinkedIn) — non</t>
-        </is>
-      </c>
+          <t>Chloe</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>P078</t>
+          <t>P079</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr">
@@ -16775,12 +16800,12 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Assemblée du 30 juin : ce que le commissaire à la transformation doit avoir remis huit jours avant</t>
+          <t>Sécurité d'un logiciel CAC : les douze questions à poser à l'éditeur</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>P2 Missions spécifiques</t>
+          <t>P3 Logiciel CAC</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -16798,7 +16823,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>P079</t>
+          <t>P080</t>
         </is>
       </c>
       <c r="B78" s="4" t="inlineStr">
@@ -16808,12 +16833,12 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Sécurité d'un logiciel CAC : les douze questions à poser à l'éditeur</t>
+          <t>Nouveautés produit de juin 2027 (à préciser)</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>P3 Logiciel CAC</t>
+          <t>P5 Produit</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -16826,12 +16851,16 @@
           <t>Chloe</t>
         </is>
       </c>
-      <c r="G78" t="inlineStr"/>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Fonctionnalités du mois identifiées — non</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>P080</t>
+          <t>P081</t>
         </is>
       </c>
       <c r="B79" s="4" t="inlineStr">
@@ -16841,12 +16870,12 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Nouveautés produit de juin 2027 (à préciser)</t>
+          <t>Paroles de commissaires aux comptes n° 9 (invité à confirmer)</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>P5 Produit</t>
+          <t>P4 Paroles de CAC</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -16861,14 +16890,14 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Fonctionnalités du mois identifiées — non</t>
+          <t>Interviewé confirmé — non</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>P081</t>
+          <t>P082</t>
         </is>
       </c>
       <c r="B80" s="4" t="inlineStr">
@@ -16878,7 +16907,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Paroles de commissaires aux comptes n° 9 (invité à confirmer)</t>
+          <t>Quatrième témoignage client (cabinet à confirmer)</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -16898,14 +16927,14 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Interviewé confirmé — non</t>
+          <t>Cabinet client volontaire identifié — non</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>P082</t>
+          <t>P083</t>
         </is>
       </c>
       <c r="B81" s="4" t="inlineStr">
@@ -16915,12 +16944,12 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Quatrième témoignage client (cabinet à confirmer)</t>
+          <t>Rafraîchissement trimestriel du panorama des logiciels CAC (T2 2027)</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>P4 Paroles de CAC</t>
+          <t>P3 Logiciel CAC</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -16933,16 +16962,12 @@
           <t>Chloe</t>
         </is>
       </c>
-      <c r="G81" t="inlineStr">
-        <is>
-          <t>Cabinet client volontaire identifié — non</t>
-        </is>
-      </c>
+      <c r="G81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>P083</t>
+          <t>P084</t>
         </is>
       </c>
       <c r="B82" s="4" t="inlineStr">
@@ -16952,12 +16977,12 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Rafraîchissement trimestriel du panorama des logiciels CAC (T2 2027)</t>
+          <t>Cycle d'été : rafraîchissement du guide IA et de la charte IA</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>P3 Logiciel CAC</t>
+          <t>P1 IA et CAC</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -16975,7 +17000,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>P084</t>
+          <t>P085</t>
         </is>
       </c>
       <c r="B83" s="4" t="inlineStr">
@@ -16985,12 +17010,12 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Cycle d'été : rafraîchissement du guide IA et de la charte IA</t>
+          <t>Cycle d'été : rafraîchissement du rapport et de la lettre de mission du commissaire aux apports</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>P1 IA et CAC</t>
+          <t>P2 Missions spécifiques</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -17008,7 +17033,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>P085</t>
+          <t>P086</t>
         </is>
       </c>
       <c r="B84" s="4" t="inlineStr">
@@ -17018,12 +17043,12 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Cycle d'été : rafraîchissement du rapport et de la lettre de mission du commissaire aux apports</t>
+          <t>Un an de blog : ce que les commissaires aux comptes nous ont demandé</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>P2 Missions spécifiques</t>
+          <t>P6 Entreprise</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -17041,7 +17066,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>P086</t>
+          <t>P087</t>
         </is>
       </c>
       <c r="B85" s="4" t="inlineStr">
@@ -17051,12 +17076,12 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Un an de blog : ce que les commissaires aux comptes nous ont demandé</t>
+          <t>Lancement de la deuxième édition du Baromètre de la formalisation</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>P6 Entreprise</t>
+          <t>Hors site</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -17074,7 +17099,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>P087</t>
+          <t>P088</t>
         </is>
       </c>
       <c r="B86" s="4" t="inlineStr">
@@ -17084,12 +17109,12 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Lancement de la deuxième édition du Baromètre de la formalisation</t>
+          <t>Nouveautés produit de juillet 2027 (à préciser)</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Hors site</t>
+          <t>P5 Produit</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -17102,12 +17127,16 @@
           <t>Chloe</t>
         </is>
       </c>
-      <c r="G86" t="inlineStr"/>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Fonctionnalités du mois identifiées — non</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>P088</t>
+          <t>P089</t>
         </is>
       </c>
       <c r="B87" s="4" t="inlineStr">
@@ -17117,12 +17146,12 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Nouveautés produit de juillet 2027 (à préciser)</t>
+          <t>Universités d'été 2027 : ce que nous présenterons aux commissaires aux comptes</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>P5 Produit</t>
+          <t>P1 IA et CAC</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -17137,14 +17166,14 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Fonctionnalités du mois identifiées — non</t>
+          <t>Participation confirmée — non</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>P089</t>
+          <t>P090</t>
         </is>
       </c>
       <c r="B88" s="4" t="inlineStr">
@@ -17154,12 +17183,12 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Universités d'été 2027 : ce que nous présenterons aux commissaires aux comptes</t>
+          <t>Paroles de commissaires aux comptes n° 10 (invité à confirmer)</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>P1 IA et CAC</t>
+          <t>P4 Paroles de CAC</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -17174,14 +17203,14 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>Participation confirmée — non</t>
+          <t>Interviewé confirmé — non</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>P090</t>
+          <t>P091</t>
         </is>
       </c>
       <c r="B89" s="4" t="inlineStr">
@@ -17191,12 +17220,12 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Paroles de commissaires aux comptes n° 10 (invité à confirmer)</t>
+          <t>Cycle d'été : rafraîchissement des articles NEP 320 et NEP 300</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>P4 Paroles de CAC</t>
+          <t>P1b NEP</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -17209,16 +17238,12 @@
           <t>Chloe</t>
         </is>
       </c>
-      <c r="G89" t="inlineStr">
-        <is>
-          <t>Interviewé confirmé — non</t>
-        </is>
-      </c>
+      <c r="G89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>P091</t>
+          <t>P092</t>
         </is>
       </c>
       <c r="B90" s="4" t="inlineStr">
@@ -17228,12 +17253,12 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Cycle d'été : rafraîchissement des articles NEP 320 et NEP 300</t>
+          <t>Cycle d'été : rafraîchissement des pages Sécurité et Équipe</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>P1b NEP</t>
+          <t>P6 Entreprise</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -17251,7 +17276,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>P092</t>
+          <t>P093</t>
         </is>
       </c>
       <c r="B91" s="4" t="inlineStr">
@@ -17261,12 +17286,12 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Cycle d'été : rafraîchissement des pages Sécurité et Équipe</t>
+          <t>Nouveautés produit de l'été 2027 (à préciser)</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>P6 Entreprise</t>
+          <t>P5 Produit</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -17279,47 +17304,14 @@
           <t>Chloe</t>
         </is>
       </c>
-      <c r="G91" t="inlineStr"/>
-    </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>P093</t>
-        </is>
-      </c>
-      <c r="B92" s="4" t="inlineStr">
-        <is>
-          <t>Idée</t>
-        </is>
-      </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>Nouveautés produit de l'été 2027 (à préciser)</t>
-        </is>
-      </c>
-      <c r="D92" t="inlineStr">
-        <is>
-          <t>P5 Produit</t>
-        </is>
-      </c>
-      <c r="E92" t="inlineStr">
-        <is>
-          <t>normale</t>
-        </is>
-      </c>
-      <c r="F92" t="inlineStr">
-        <is>
-          <t>Chloe</t>
-        </is>
-      </c>
-      <c r="G92" t="inlineStr">
+      <c r="G91" t="inlineStr">
         <is>
           <t>Fonctionnalités identifiées — non</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G92"/>
+  <autoFilter ref="A1:G91"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Publication de l'article « NEP 911 et 912 révisées » : indexation, sitemap, flux, llms.txt
Brief P011 passé en statut Publié après accord de Chloe (feuille Décisions).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content-plan/plan-editorial.xlsx
+++ b/content-plan/plan-editorial.xlsx
@@ -43,7 +43,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -65,11 +65,6 @@
         <fgColor rgb="00EEEEEE"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFE699"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -83,7 +78,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -91,7 +86,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1594,9 +1588,9 @@
           <t>P011</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Relecture humaine</t>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Publié</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1642,8 +1636,16 @@
           <t>2026-09-29</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>https://checkia.fr/blog/futur-de-l-audit/nep-911-912-revisees-2026/</t>
+        </is>
+      </c>
       <c r="P12" t="inlineStr">
         <is>
           <t>haute</t>
@@ -1681,7 +1683,7 @@
       </c>
       <c r="AA12" t="inlineStr">
         <is>
-          <t>non</t>
+          <t>oui</t>
         </is>
       </c>
     </row>
@@ -11331,7 +11333,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Relecture humaine</t>
+          <t>Publié</t>
         </is>
       </c>
     </row>
@@ -13091,10 +13093,14 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Relecture humaine</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
+          <t>Publié</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>https://checkia.fr/blog/futur-de-l-audit/nep-911-912-revisees-2026/</t>
+        </is>
+      </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
@@ -13966,7 +13972,11 @@
           <t>https://checkia.fr/blog/futur-de-l-audit/nep-911-912-revisees-2026/</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>

</xml_diff>

<commit_message>
Plan éditorial : les articles « logiciel CAC » passent dans Le futur de l'audit
Nouveautés produit ne contient plus que les fonctionnalités livrées.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content-plan/plan-editorial.xlsx
+++ b/content-plan/plan-editorial.xlsx
@@ -1735,7 +1735,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Nouveautés produit</t>
+          <t>Le futur de l'audit</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
@@ -2414,7 +2414,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Nouveautés produit</t>
+          <t>Le futur de l'audit</t>
         </is>
       </c>
       <c r="F21" t="inlineStr"/>
@@ -3405,7 +3405,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Nouveautés produit</t>
+          <t>Le futur de l'audit</t>
         </is>
       </c>
       <c r="F32" t="inlineStr"/>
@@ -4716,7 +4716,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Nouveautés produit</t>
+          <t>Le futur de l'audit</t>
         </is>
       </c>
       <c r="F47" t="inlineStr"/>
@@ -5517,7 +5517,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Nouveautés produit</t>
+          <t>Le futur de l'audit</t>
         </is>
       </c>
       <c r="F56" t="inlineStr"/>
@@ -6322,7 +6322,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Nouveautés produit</t>
+          <t>Le futur de l'audit</t>
         </is>
       </c>
       <c r="F65" t="inlineStr"/>
@@ -7026,7 +7026,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Nouveautés produit</t>
+          <t>Le futur de l'audit</t>
         </is>
       </c>
       <c r="F73" t="inlineStr"/>
@@ -8430,7 +8430,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Nouveautés produit</t>
+          <t>Le futur de l'audit</t>
         </is>
       </c>
       <c r="F89" t="inlineStr"/>

</xml_diff>